<commit_message>
added fragmentation test data
</commit_message>
<xml_diff>
--- a/data/test_samples/static/output_graph/hazard_names.xlsx
+++ b/data/test_samples/static/output_graph/hazard_names.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>GHG_timesteps_test1</t>
+          <t>Frag_timesteps_test1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -468,14 +468,14 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_hazard_timesteps\GHG_timesteps_test1.tif</t>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test1.tif</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GHG_timesteps_test1</t>
+          <t>Frag_timesteps_test1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -490,14 +490,14 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_hazard_timesteps\GHG_timesteps_test1.tif</t>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test1.tif</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>GHG_timesteps_test2</t>
+          <t>Frag_timesteps_test2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -512,14 +512,14 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_hazard_timesteps\GHG_timesteps_test2.tif</t>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test2.tif</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GHG_timesteps_test2</t>
+          <t>Frag_timesteps_test2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -534,14 +534,14 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_hazard_timesteps\GHG_timesteps_test2.tif</t>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test2.tif</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GHG_timesteps_test3</t>
+          <t>Frag_timesteps_test3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -556,14 +556,14 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_hazard_timesteps\GHG_timesteps_test3.tif</t>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test3.tif</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>GHG_timesteps_test3</t>
+          <t>Frag_timesteps_test3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -578,14 +578,14 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_hazard_timesteps\GHG_timesteps_test3.tif</t>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test3.tif</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>GHG_timesteps_test4</t>
+          <t>Frag_timesteps_test4</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -600,14 +600,14 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_hazard_timesteps\GHG_timesteps_test4.tif</t>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test4.tif</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GHG_timesteps_test4</t>
+          <t>Frag_timesteps_test4</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -622,14 +622,14 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_hazard_timesteps\GHG_timesteps_test4.tif</t>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test4.tif</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GHG_timesteps_test5</t>
+          <t>Frag_timesteps_test5</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -644,14 +644,14 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_hazard_timesteps\GHG_timesteps_test5.tif</t>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test5.tif</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GHG_timesteps_test5</t>
+          <t>Frag_timesteps_test5</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -666,7 +666,183 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>C:\repos\powerpath\data\test_samples\test_hazard_timesteps\GHG_timesteps_test5.tif</t>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test5.tif</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Frag_timesteps_test6</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>maximum</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>EV6_ma</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test6.tif</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Frag_timesteps_test6</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>fraction of network segment impacted by hazard</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>EV6_fr</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test6.tif</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Frag_timesteps_test7</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>maximum</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>EV7_ma</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test7.tif</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Frag_timesteps_test7</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>fraction of network segment impacted by hazard</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>EV7_fr</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test7.tif</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Frag_timesteps_test8</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>maximum</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>EV8_ma</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test8.tif</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Frag_timesteps_test8</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>fraction of network segment impacted by hazard</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>EV8_fr</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test8.tif</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Frag_timesteps_test9</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>maximum</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>EV9_ma</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test9.tif</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Frag_timesteps_test9</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>fraction of network segment impacted by hazard</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>EV9_fr</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>C:\repos\powerpath\data\test_samples\test_fragmentation\Frag_timesteps_test9.tif</t>
         </is>
       </c>
     </row>

</xml_diff>